<commit_message>
fix: header area_id y carrera_id
</commit_message>
<xml_diff>
--- a/Scripts/layouts/oferta_academicav2.2.xlsx
+++ b/Scripts/layouts/oferta_academicav2.2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emanu\Documents\Athena\Scripts\layouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C75095C-9536-4F89-869A-EBD8D5BD49C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34C8AE20-C1AE-4B42-A126-FC114D303F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="area" sheetId="4" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: carrera y area en header
</commit_message>
<xml_diff>
--- a/Scripts/layouts/oferta_academicav2.2.xlsx
+++ b/Scripts/layouts/oferta_academicav2.2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emanu\Documents\Athena\Scripts\layouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34C8AE20-C1AE-4B42-A126-FC114D303F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C64CC042-DC97-4156-90CF-B0444FF060A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2105,7 +2105,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2154,6 +2154,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor rgb="FF2F5496"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -2197,7 +2203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2249,6 +2255,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2843,7 +2852,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="19" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="18" t="s">

</xml_diff>